<commit_message>
Added separate column for segment widths
</commit_message>
<xml_diff>
--- a/AnthropometricTableComplete.xlsx
+++ b/AnthropometricTableComplete.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\draga\mujoco-biomechanics\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F274228-A7F2-406E-B4AE-0E19D851BBA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11580" activeTab="1"/>
+    <workbookView xWindow="-28905" yWindow="1665" windowWidth="14610" windowHeight="15585" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Male" sheetId="1" r:id="rId1"/>
@@ -28,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="39">
   <si>
     <t>Body Part</t>
   </si>
@@ -146,20 +152,19 @@
   </si>
   <si>
     <t>35i</t>
+  </si>
+  <si>
+    <t>Segment width</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="0.0_ "/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="0.0_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -189,353 +194,16 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="33">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="9">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -543,251 +211,9 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="49">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -801,66 +227,22 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="178" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="49">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="1" builtinId="3"/>
-    <cellStyle name="Currency" xfId="2" builtinId="4"/>
-    <cellStyle name="Percent" xfId="3" builtinId="5"/>
-    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
-    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
-    <cellStyle name="Link" xfId="6" builtinId="8"/>
-    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
-    <cellStyle name="Note" xfId="8" builtinId="10"/>
-    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
-    <cellStyle name="Title" xfId="10" builtinId="15"/>
-    <cellStyle name="CExplanatory Text" xfId="11" builtinId="53"/>
-    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
-    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
-    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
-    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
-    <cellStyle name="Input" xfId="16" builtinId="20"/>
-    <cellStyle name="Output" xfId="17" builtinId="21"/>
-    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
-    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
-    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
-    <cellStyle name="Total" xfId="21" builtinId="25"/>
-    <cellStyle name="Good" xfId="22" builtinId="26"/>
-    <cellStyle name="Bad" xfId="23" builtinId="27"/>
-    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
-    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
-    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
-    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
-    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
-    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
-    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
-    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
-    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
-    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
-    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
-    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
-    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
-    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
-    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
-    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
-    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
-    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
-    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
-    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
-    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
-    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
-    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
-    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
-    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1118,22 +500,22 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="10.6666666666667" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.8666666666667" customWidth="1"/>
-    <col min="2" max="2" width="19.4666666666667" customWidth="1"/>
-    <col min="3" max="3" width="20.8" customWidth="1"/>
-    <col min="4" max="6" width="15.8" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" customWidth="1"/>
+    <col min="2" max="2" width="19.453125" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" customWidth="1"/>
+    <col min="4" max="6" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="100.05" customHeight="1" spans="1:12">
+    <row r="1" spans="1:12" ht="100" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1171,12 +553,12 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" ht="50" customHeight="1" spans="1:12">
+    <row r="2" spans="1:12" ht="50" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4">
-        <v>0.139</v>
+        <v>0.13900000000000001</v>
       </c>
       <c r="C2" s="4">
         <v>1.2</v>
@@ -1185,7 +567,7 @@
         <v>50.2</v>
       </c>
       <c r="E2" s="4">
-        <v>-19.9</v>
+        <v>-19.899999999999999</v>
       </c>
       <c r="F2" s="4">
         <v>3.4</v>
@@ -1209,7 +591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="50" customHeight="1" spans="1:12">
+    <row r="3" spans="1:12" ht="50" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
@@ -1247,7 +629,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" ht="50" customHeight="1" spans="1:12">
+    <row r="4" spans="1:12" ht="50" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -1258,7 +640,7 @@
         <v>12.3</v>
       </c>
       <c r="D4" s="4">
-        <v>-4.1</v>
+        <v>-4.0999999999999996</v>
       </c>
       <c r="E4" s="4">
         <v>-42.9</v>
@@ -1285,7 +667,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" ht="50" customHeight="1" spans="1:12">
+    <row r="5" spans="1:12" ht="50" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
@@ -1296,7 +678,7 @@
         <v>0.6</v>
       </c>
       <c r="D5" s="4">
-        <v>8.2</v>
+        <v>8.1999999999999993</v>
       </c>
       <c r="E5" s="4">
         <v>-83.9</v>
@@ -1323,12 +705,12 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" ht="50" customHeight="1" spans="1:12">
+    <row r="6" spans="1:12" ht="50" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
       <c r="B6" s="4">
-        <v>0.283</v>
+        <v>0.28299999999999997</v>
       </c>
       <c r="C6" s="4">
         <v>1.7</v>
@@ -1340,7 +722,7 @@
         <v>-41.7</v>
       </c>
       <c r="F6" s="4">
-        <v>1.1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="G6" s="4">
         <v>28</v>
@@ -1361,12 +743,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" ht="50" customHeight="1" spans="1:12">
+    <row r="7" spans="1:12" ht="50" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>23</v>
       </c>
       <c r="B7" s="4">
-        <v>0.277</v>
+        <v>0.27700000000000002</v>
       </c>
       <c r="C7" s="4">
         <v>2.4</v>
@@ -1399,12 +781,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" ht="50" customHeight="1" spans="1:12">
+    <row r="8" spans="1:12" ht="50" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B8" s="4">
-        <v>0.093</v>
+        <v>9.2999999999999999E-2</v>
       </c>
       <c r="C8" s="4">
         <v>14.2</v>
@@ -1437,7 +819,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="9" ht="50" customHeight="1" spans="1:12">
+    <row r="9" spans="1:12" ht="50" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
@@ -1448,7 +830,7 @@
         <v>2.9</v>
       </c>
       <c r="D9" s="4">
-        <v>17.6</v>
+        <v>17.600000000000001</v>
       </c>
       <c r="E9" s="4">
         <v>-36.1</v>
@@ -1475,12 +857,12 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" ht="50" customHeight="1" spans="1:12">
+    <row r="10" spans="1:12" ht="50" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="4">
-        <v>0.334</v>
+        <v>0.33400000000000002</v>
       </c>
       <c r="C10" s="4">
         <v>30.4</v>
@@ -1513,12 +895,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="11" ht="50" customHeight="1" spans="1:12">
+    <row r="11" spans="1:12" ht="50" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="4">
-        <v>0.278</v>
+        <v>0.27800000000000002</v>
       </c>
       <c r="C11" s="4">
         <v>6.7</v>
@@ -1554,23 +936,21 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:L11"/>
-  <sheetFormatPr defaultColWidth="10.6666666666667" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultColWidth="10.6328125" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="19.8666666666667" customWidth="1"/>
-    <col min="2" max="2" width="19.4666666666667" customWidth="1"/>
-    <col min="3" max="3" width="20.8" customWidth="1"/>
-    <col min="4" max="6" width="15.8" customWidth="1"/>
+    <col min="1" max="1" width="19.81640625" customWidth="1"/>
+    <col min="2" max="2" width="18.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.81640625" customWidth="1"/>
+    <col min="4" max="6" width="15.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="100.05" customHeight="1" spans="1:12">
+    <row r="1" spans="1:13" ht="100" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1607,19 +987,22 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" ht="50" customHeight="1" spans="1:12">
+      <c r="M1" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="50" customHeight="1">
       <c r="A2" s="4" t="s">
         <v>12</v>
       </c>
       <c r="B2" s="4">
-        <v>0.117</v>
+        <v>0.11700000000000001</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4">
-        <v>38.2</v>
+        <v>38.200000000000003</v>
       </c>
       <c r="E2" s="4">
         <v>-30.9</v>
@@ -1645,19 +1028,22 @@
       <c r="L2" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="3" ht="50" customHeight="1" spans="1:12">
+      <c r="M2" s="6">
+        <v>0.10100000000000001</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="50" customHeight="1">
       <c r="A3" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B3" s="4">
-        <v>0.388</v>
+        <v>0.38800000000000001</v>
       </c>
       <c r="C3" s="4">
         <v>4.5</v>
       </c>
       <c r="D3" s="4">
-        <v>-4.9</v>
+        <v>-4.9000000000000004</v>
       </c>
       <c r="E3" s="4">
         <v>-40.4</v>
@@ -1683,8 +1069,11 @@
       <c r="L3" s="6">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" ht="50" customHeight="1" spans="1:12">
+      <c r="M3" s="6">
+        <v>0.10299999999999999</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="50" customHeight="1">
       <c r="A4" s="4" t="s">
         <v>17</v>
       </c>
@@ -1698,7 +1087,7 @@
         <v>-7.7</v>
       </c>
       <c r="E4" s="4">
-        <v>-37.7</v>
+        <v>-37.700000000000003</v>
       </c>
       <c r="F4" s="4">
         <v>0.8</v>
@@ -1721,13 +1110,16 @@
       <c r="L4" s="6" t="s">
         <v>18</v>
       </c>
-    </row>
-    <row r="5" ht="50" customHeight="1" spans="1:12">
+      <c r="M4" s="6">
+        <v>0.16300000000000001</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="50" customHeight="1">
       <c r="A5" s="4" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="4">
-        <v>0.071</v>
+        <v>7.0999999999999994E-2</v>
       </c>
       <c r="C5" s="4">
         <v>0.5</v>
@@ -1759,8 +1151,11 @@
       <c r="L5" s="6" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="6" ht="50" customHeight="1" spans="1:12">
+      <c r="M5" s="6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="50" customHeight="1">
       <c r="A6" s="4" t="s">
         <v>21</v>
       </c>
@@ -1797,8 +1192,11 @@
       <c r="L6" s="6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" ht="50" customHeight="1" spans="1:12">
+      <c r="M6" s="6">
+        <v>8.5999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="50" customHeight="1">
       <c r="A7" s="4" t="s">
         <v>23</v>
       </c>
@@ -1806,7 +1204,7 @@
         <v>0.251</v>
       </c>
       <c r="C7" s="4">
-        <v>2.3</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D7" s="4">
         <v>-5.5</v>
@@ -1835,13 +1233,16 @@
       <c r="L7" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" ht="50" customHeight="1" spans="1:12">
+      <c r="M7" s="6">
+        <v>0.10100000000000001</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" ht="50" customHeight="1">
       <c r="A8" s="4" t="s">
         <v>25</v>
       </c>
       <c r="B8" s="4">
-        <v>0.103</v>
+        <v>0.10299999999999999</v>
       </c>
       <c r="C8" s="4">
         <v>14.7</v>
@@ -1873,8 +1274,11 @@
       <c r="L8" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" ht="50" customHeight="1" spans="1:12">
+      <c r="M8" s="6">
+        <v>0.28100000000000003</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="50" customHeight="1">
       <c r="A9" s="4" t="s">
         <v>29</v>
       </c>
@@ -1882,7 +1286,7 @@
         <v>0.125</v>
       </c>
       <c r="C9" s="4">
-        <v>4.1</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="D9" s="4">
         <v>21.9</v>
@@ -1911,13 +1315,16 @@
       <c r="L9" s="6" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="10" ht="50" customHeight="1" spans="1:12">
+      <c r="M9" s="6">
+        <v>0.27600000000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="50" customHeight="1">
       <c r="A10" s="4" t="s">
         <v>32</v>
       </c>
       <c r="B10" s="4">
-        <v>0.322</v>
+        <v>0.32200000000000001</v>
       </c>
       <c r="C10" s="4">
         <v>26.3</v>
@@ -1949,13 +1356,16 @@
       <c r="L10" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" ht="50" customHeight="1" spans="1:12">
+      <c r="M10" s="6">
+        <v>0.30099999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="50" customHeight="1">
       <c r="A11" s="4" t="s">
         <v>33</v>
       </c>
       <c r="B11" s="4">
-        <v>0.243</v>
+        <v>0.24299999999999999</v>
       </c>
       <c r="C11" s="4">
         <v>6.7</v>
@@ -1985,12 +1395,14 @@
         <v>1</v>
       </c>
       <c r="L11" s="6">
+        <v>0</v>
+      </c>
+      <c r="M11" s="6">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>